<commit_message>
Stage 2-1c：CAP_008／011、HW_040 讀到原文，HW_014、DEM_011 登錄，E2 Rubin Ultra 單架 72 候選
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KztG65vgqgX1BbzRnjYqk7
</commit_message>
<xml_diff>
--- a/docs/reports/20261005_stage2-1_查核.xlsx
+++ b/docs/reports/20261005_stage2-1_查核.xlsx
@@ -19,6 +19,8 @@
     <sheet name="SRC格敏感度（查核佇列）" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="1b 影響計算" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="1b 判讀與阻擋清單" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="1c 查核結果" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="1c E2 Rubin Ultra 單架72" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'查核紀錄'!$A$1:$T$30</definedName>
@@ -448,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -596,6 +598,18 @@
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>新增查核 SRC_CAP_008／011、SRC_HW_025／028；補讀 SRC_HW_047（GB200、VR200）與 SRC_HW_001（DGX H100／H200 使用手冊）；新增『1b 影響計算』『1b 判讀與阻擋清單』；『查核紀錄』更新並附 4 列，『待 Project 判斷』附 6 項。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>1c（2026-10-05）</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>網路重測：artificialanalysis.ai HTTP 200、www.nvidia.com HTTP 307→200（非 403）。新增頁「1c 查核結果」「1c E2 Rubin Ultra 單架72」；更新「查核紀錄」（CAP_008／011、HW_040、HW_014、DEM_011）與「待 Project 判斷」。supermicro.com、flex.com、blog.se.com、prnewswire.com、storagereview.com、semianalysis.com 等仍為出口政策 CONNECT 403，未繞過。</t>
         </is>
       </c>
     </row>
@@ -21928,6 +21942,936 @@
       <c r="D15" s="2" t="inlineStr">
         <is>
           <t>https://www.wing.vc/content/how-much-does-an-nvidia-nvl72-cost；tomshardware.com（原報導網址見 SRC 出處欄）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>SRC_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>讀取結果</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>原文摘錄／換算</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>與現值</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>建議等級</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>立場</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SRC_CAP_008</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>AA Intelligence Index v4.3.2：GPT-6 Sol (Max)＝48</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>R1（artificialanalysis.ai，HTTP 200）</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>表列 Intelligence Index：48｜45；頁面註明 v4.3.2</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>一致</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>中立（評測集與權重由 AA 自訂）</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>升級候選；敏感度最高</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SRC_CAP_011</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>GLM-5.3 (Max)＝45</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>R1（同頁）</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>一致</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>升級候選</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_040</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>H100 FP8 dense 1.979 PF</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>R1（nvidia.com/en-us/data-center/h100/，HTTP 200）</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>FP8 Tensor Core * 3,958 teraFLOPS；* With sparsity；÷2＝1,979</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>一致（換算）</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1（Derived）</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Interested-party（NVIDIA 為賣方）</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>前輪「值不同」撤回；原文未直接寫 dense 值</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_014</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>VR NVL72 機架功率 227 kW</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>R1（Schneider 部落格，chat 端已讀；CC 環境 CONNECT 403）</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>MaxQ 188 kW／MaxP 227 kW per rack（參考設計）</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>一致（F9）；F8 190 對 188、F10 230 對 227 待判斷</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Interested-party：供電與冷卻設備商</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>原「Supermicro DLC-2 設計點」出處更正；Supermicro 新聞稿全文無 227 kW（Andy 已讀）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_014 佐證</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Supermicro SRS-VR-NVL72 Datasheet（G2，Andy 提供）</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>R1（Andy 提供）</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>4×3U 110 kW 電源架＝440 kW［Verified，含備援］；In-Row CDU 2.2 MW／8 架＝275 kW/架［Derived］</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>227 &lt; 275 &lt; 440，不衝突</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>—（佐證）</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Interested-party（系統廠）</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>備援配置（N+N／N+1）之查詢已取消。僅註記：搜尋摘錄（SemiAnalysis，R5 未讀）稱 4×110 kW 供 ≤220 kW，若屬實則可用容量低於 MaxP 227，未驗證</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SRC_DEM_011</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI API &gt;15 B tok/min（2026-03-31）</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>R1（Andy 提供，G2；繁中官方頁）</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>「我們的 API 目前每分鐘可處理超過 150 億個 Token。」</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>一致</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Interested-party（融資公告；誘因＝呈現規模成長）</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>繁中譯本；時點值；「超過」為下界</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="64" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Spec_Rack 格</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>現值（Kyber 144 封裝／架）</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>新定義（單架 72 GPU）候選值</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>計算與出處</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>讀取結果</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>標記</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>待判斷或備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>定義</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>G4／G5／G19</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rubin Ultra NVL576（Kyber）；註：GPU 數為封裝數，144 封裝＝576 die</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>「Rubin Ultra（MGX NVL 單架，72 GPU）」；NVL576＝8 架互連</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA 技術部落格（2026-09）：“Vera Rubin Ultra NVL576 will combine eight separate MGX NVL racks, each with 72 Rubin Ultra GPUs, all in a single 576-GPU NVLink domain”；Kyber NVL144 另列 “double the NVLink domain per rack to 144 GPUs for the Feynman era”</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>R1 已讀原文（developer.nvidia.com/blog/nvidia-vera-rubin-pod-seven-chips-five-rack-scale-systems-one-ai-supercomputer）</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>「GPU」在新稿是封裝或 die 未明載。推斷（Derived）：封裝，因 Kyber NVL144＝144 封裝＝舊 NVL576（576 die）；若 72 指 die 則單架僅 18 封裝，與 MGX 單架 72 GPU 的描述不合。需 Project 確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>G6 GPU 封裝／架</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>G6 =SRC_HW_054</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA 同上（“each with 72 Rubin Ultra GPUs”）；SRC_HW_054 現值 144 屬 Kyber，不再適用單架</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Verified（NVIDIA 官方，Interested-party）</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>新增 SRC 或改引 NVIDIA 部落格；SRC_HW_054 保留給 Kyber 備查</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>G28 Scale-up 域 GPU 數</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>G28 =SRC_HW_054</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>兩種讀法：72（單架）或 576（NVL576 域，兩層 NVLink）</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>同上：“single 576-GPU NVLink domain”</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>模型用 G28 作 EP 通訊域寬度；單架內全互連為 72，跨 8 架為兩層拓撲（頻寬不同）。Project 判斷取 72 或 576</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>G8／G9／G10 功率 低／基準／高（kW/架）</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>G8 550／G9 =SRC_HW_013（600）／G10 650</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>550／600／650（Kyber 單架）</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>(a) 按封裝數比例 300（低約 270、高約 325）［Derived：600×72/144；每 GPU 4.17 kW 與現值相同］；(b) 按 VR 比值：GPU 3.6 kW×72＝259 kW，×(227/(72×1.8))＝1.75 → 約 454 kW［Derived，Analogy］</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA 官方未公布單架功率（部落格查無 kW）；800 VDC 部落格僅稱可由 100 kW 到 &gt;1 MW 機架；舊值 600 kW 出自 DCD 等二手（SRC_HW_013，3 級）</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>R1 讀到 NVIDIA 部落格但無數值；功率候選為 Derived／Analogy</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Derived／Assumed：以區間呈現，不提議基準</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>範圍約 300–454 kW。取 (a) 則每 GPU 功率與現行不變，單架絕對值減半；取 (b) 較貼近 VR 世代 MaxP／GPU 功率比（1.75）。Project 決定</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>G11／G12／G13 價格 低／基準／高（$M/架）</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>23.4／31.2／39</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>VR 每 GPU 價 7.8/72＝0.1083 $M ×1.5／2.0／2.5×144</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>72 GPU：11.7／15.6／19.5（同公式，封裝減半）</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>公式為現行 Assumed 推估（G14 註）；無公開報價</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>無一手來源（R6：以「Rubin Ultra rack price」「Rubin Ultra price per GPU」查詢，僅見推估，未入帳）</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Assumed</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>倍數 1.5／2.0／2.5 本身即 Assumed；單架價與每 GPU 價隨封裝數線性，不新增資訊</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>G23 峰值 dense（基準）PF/GPU</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>G23</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>70（＝2×VR NVFP4 訓練 dense 35）［Derived］</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA DGX VR NVL72 頁：NVFP4 Training 2,520 PFLOPS（72 GPU＝35／GPU），註 “**Dense specification”；Rubin Ultra 為 4 die（Rubin 2 die）</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>R1（VR 原文）＋Derived（×2）</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>現值 73 的來源未在此重查（現行標 Assumed）；候選 70 與 73 差 4%。RU 規格 NVIDIA 未直接公布每 GPU NVFP4 dense</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>G24 峰值高情境 NVFP4 推論 PF/GPU</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>G24</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>104（15 EF÷144）</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA 路線圖：Rubin Ultra 每封裝 100 PF FP4（搜尋摘錄，Tom's Hardware 等；R5 未讀原文）；VR 頁 NVFP4 推論 50 PF/GPU 註 “Sparse specification”，100＝2×50 一致</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>搜尋摘錄（R5）＋Derived 交叉</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Analogy／Interested-party</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>每封裝值不隨機架定義改變；104 與 100 差 4%（15 EF／144＝104.2 對 100 PF）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>G25 HBM 容量 GB/GPU</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>G25</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>1024</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>1024（不變；每封裝 1 TB HBM4e）</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>搜尋摘錄（R5）；VR 單 GPU 288 GB 為 NVIDIA 部落格 R1</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Analogy</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>每封裝值，不因單架改變</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>G26 HBM 頻寬 TB/s/GPU</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>G26</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>32（不變；舊 4.6 PB/s÷144＝31.9）</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>搜尋摘錄（R5）</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Analogy</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>每封裝值不變</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>G33 GPU 功率 W/封裝</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>G33</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>3600</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>3600（不變）；單架 GPU 合計 259 kW</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Assumed（RU 推估）</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Assumed</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>每封裝值不變</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>G40 FP8 dense 訓練 PF/GPU</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>G40 =SRC_HW_045 → 34.7</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>34.7（5 EF÷144）</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>34.7（不變）；交叉：VR FP8/FP6 訓練 dense 17.5 PF/GPU（2 die）×2＝35.0［Derived］，與 34.7 差 0.9%</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA DGX VR NVL72 頁：FP8/FP6 Training 1,260 PFLOPS＝17.5／GPU，註 “**Dense specification”（R1）；舊值 5 EF 來自 NVIDIA 路線圖（二手轉載）</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>R1（VR 原文）＋Derived</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>證據支持 34.7 為 dense 口徑（前輪列「未讀原文，間接證據」），SRC_HW_045 值 5000 PF 是整機，每封裝＝5000/144；改單架後 SRC_HW_045 需改為每封裝值或單架 2,500 PF（72×34.7）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>其他 G 欄格（G39、G41、G27、G29–G32、G34–G36）</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>8／73／1.8／64／0.5625／1／8／18／公式</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>隨每封裝規格不變；唯 G27 EP 頻寬、G29 EP 寬度、G32 prefill 實例若依單架 72 GPU 重新定義，屬公式輸入，需 Project 判斷</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>G14 文字（144 封裝；價格＝VR×1.5–2.5）、G15 功率來源（約 600 kW）、G16、G17 標記（Assumed）需同步改寫</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>不納入</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Kyber NVL144（144 GPU／架）</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA 同篇：Feynman 時代</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>依 Andy 決定不納入；Schneider 稱 Rubin Ultra＝Kyber 576 GPU／架、1–1.2 MW，與 NVIDIA 2026-09 衝突，列較舊路線圖，以 NVIDIA 為準</t>
         </is>
       </c>
     </row>
@@ -23951,7 +24895,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Supermicro VR NVL72 散熱設計點</t>
+          <t>VR NVL72 MaxP 機架功率（原記 Supermicro DLC-2 設計點）</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -23974,50 +24918,50 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://ir.supermicro.com/news/news-details/2026/Supermicro-Now-Shipping-NVIDIA-Vera-Rubin-NVL72-Racks/default.aspx（SRC 現引 windowsforum.com 轉述）</t>
+          <t>https://blog.se.com/datacenter/2026/05/08/nvidia-and-schneider-electric-get-in-sync-at-nvidia-gtc-2026-to-deliver-vera-rubin-ai-factories/（Schneider Electric 部落格，2026-05-08；chat 端已讀原文）</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-05（chat 端讀取，Andy 提供）</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（ir.supermicro.com HTTP 403，WAF 擋 CLI）；僅見搜尋摘要</t>
+          <t>R1 已讀原文（chat 端；CC 本環境 blog.se.com CONNECT 403，未獨立讀，依指令登錄；G2）</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>VR NVL72 參考設計支援 MaxQ 188 kW/rack、MaxP 227 kW/rack（依 chat 端轉述，非 CC 逐字摘錄）</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>搜尋摘要：DLC-2「sized for 227 kW per rack」（Supermicro 新聞稿）</t>
+          <t>MaxP 227 kW；MaxQ 188 kW</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>—（散熱設計點，非 NVIDIA 官方機架功率）</t>
+          <t>無需換算；口徑＝機架 MaxP（參考設計；IT 側，非設施）</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>一致（依搜尋摘要）</t>
+          <t>一致（F9＝227）；F8 低 190 對 MaxQ 188（−1.1%）、F10 高 230 對 MaxP 227 另列判斷</t>
         </is>
       </c>
       <c r="N7" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>利害關係方：Supermicro 為系統廠；散熱「設計」上限偏保守（誘因：展示散熱能力）</t>
+          <t>Interested-party：Schneider Electric 為供電與冷卻設備商，誘因＝展示其設計可承載的 VR 機架</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>無（NVIDIA 官方 VR200 NVL72 機架功率未找到）</t>
+          <t>佐證（G2，Andy 提供）：Supermicro〈Supermicro NVIDIA Vera Rubin NVL72〉Datasheet（SRS-VR-NVL72，© 2026）：4×3U 110 kW 電源架（裝置容量 440 kW［Verified，含備援］）；In-Row CDU 最高 2.2 MW、支援最多 8 架（每架冷卻上限 275 kW［Derived］）。另 Supermicro 2026-09-23 新聞稿（Andy 已讀）全文無 227 kW。非獨立於 NVIDIA 參考設計，為不同設備商的容量上限，與 227 kW 不衝突（227 &lt; 275 &lt; 440）。</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
@@ -24027,7 +24971,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>已知一手網址（Supermicro 新聞稿）；Andy 可提供原文</t>
+          <t>1c：原 SRC 記「Supermicro DLC-2 設計點」，經 Andy 讀新聞稿確認該稿無 227 kW；實際出處改為 Schneider 部落格（NVIDIA 參考設計 MaxP）。標籤文字（Spec_Rack F15「Supermicro DLC-2 設計點 227 kW（S8）」）需 v5.18 更正，屬判斷類，交 Project。CC 的搜尋摘要曾見 Supermicro 產品頁稱 “sized for 227 kW per rack”（supermicro.com 被擋，未讀原文，R5；僅旁證，不作依據）。查電源架備援配置之工作已取消。</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -24037,7 +24981,7 @@
       </c>
       <c r="T7" s="2" t="inlineStr">
         <is>
-          <t>只見搜尋摘錄 → 3 級</t>
+          <t>一手設備商原文（chat 端已讀）→ 1 級；利害關係方立場另欄</t>
         </is>
       </c>
     </row>
@@ -24562,7 +25506,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>https://developer.nvidia.com/blog/inside-nvidia-blackwell-ultra-the-chip-powering-the-ai-factory-era/；https://developer.nvidia.com/blog/nvidia-hopper-architecture-in-depth/（nvidia.com 規格表被封鎖）</t>
+          <t>https://www.nvidia.com/en-us/data-center/h100/（1c 新增；前輪為 developer.nvidia.com 部落格）</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -24572,31 +25516,31 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R1 已讀原文（一手；NVIDIA 技術部落格表格）：但只給進位值；精確值 1.979 的規格表 R5 被封鎖</t>
+          <t>R1 已讀原文（一手；nvidia.com 規格表，1c 重讀，HTTP 200）</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>“FP8 dense | sparse performance 2 | 4 PetaFLOPS”（Hopper 欄）</t>
+          <t>“FP8 Tensor Core * 3,958 teraFLOPS”（SXM）；表末註 “* With sparsity”；BF16／FP16 同列 1,979（含稀疏）</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2（PF，進位）；Hopper 白皮書表為 2000 | 4000 TFLOPS</t>
+          <t>3,958 TFLOPS（含稀疏，SXM）</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>現值 1.979 對 2.0：−1.05%（原文進位）</t>
+          <t>dense＝含稀疏值 ÷2＝3,958÷2＝1,979 TFLOPS＝1.979 PF（NVIDIA 慣例；交叉：BF16 1,979÷2＝989.5≈SRC 0.989 的 BF16 列）</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>不一致（進位值 2.0 對 1.979，容差 0 不符）；口徑（dense）相同</t>
+          <t>一致（換算後相同，容差 0；前輪「值不同」結論撤回——前輪只讀到進位值 2）</t>
         </is>
       </c>
       <c r="N13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -24615,7 +25559,7 @@
       </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>S1：值不同（進位）→ 交 Andy。1.979 為 NVIDIA 資料表常見寫法（3,958 稀疏的一半），本次未讀到該表</t>
+          <t>1c：由 R3→R1，S1 (a) 升級候選（附換算式；原文未直接寫「dense 1,979」，÷2 為 NVIDIA 慣例，標 [Derived]）。僅讀 SXM 欄；PCIe 欄 3,341 含稀疏不適用。</t>
         </is>
       </c>
       <c r="S13" s="2" t="inlineStr">
@@ -24625,7 +25569,7 @@
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
-          <t>一手已讀但值未能核對到 1.979 → 維持 3 級</t>
+          <t>一手原文已讀；換算後值相同 → 1 級（Derived）</t>
         </is>
       </c>
     </row>
@@ -26130,45 +27074,45 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>https://openai.com/index/accelerating-the-next-phase-ai/（HTTP 403）</t>
+          <t>https://openai.com/zh-Hant/index/accelerating-the-next-phase-ai/（OpenAI 繁中頁；Andy 已讀；CC 本環境 openai.com HTTP 403 網站本身阻擋）</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-05（Andy 讀取，提供給 CC）</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（openai.com HTTP 403，WAF 擋 CLI；鏡像站依規則不繞過）；僅見搜尋摘要</t>
+          <t>R1 已讀原文（Andy 提供；G2）。OpenAI 官方繁中頁，2026-03-31</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>「我們的 API 目前每分鐘可處理超過 150 億個 Token。」</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>搜尋摘要：融資公告稱 API 平台目前每分鐘處理「超過 150 億 token」（2026-03 融資 $122B、估值 $852B）</t>
+          <t>&gt; 15 B tok/min（150 億）</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>無需換算（150 億＝15 B）</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>一致（數值；依搜尋摘要）；時點不明：不同轉述寫「2025 年底」「2026-04」，並有一則稱 2025-10 為 6B tok/min、2026-04 為 15B</t>
+          <t>一致（值、「超過」用語、口徑＝OpenAI API、時點 2026-03-31）</t>
         </is>
       </c>
       <c r="N29" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>利害關係方：OpenAI 融資公告，有呈現成長的誘因</t>
+          <t>Interested-party：OpenAI 融資公告，有呈現成長與規模的誘因</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -26183,7 +27127,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取。搜尋摘要仍稱 API「超過 150 億 token／分」，並有說法稱 2025-10 為 60 億、2026-04 為 150 億（時點仍需原文）；現等級 2 建議降為 3 或待讀（交 Andy）</t>
+          <t>1c：由 R5→R1（Andy 提供）。限制：讀的是繁中譯本，非英文原文；若需逐字英文可另請 Andy 提供。時點值（融資公告當時），非 2026-10 現值。「超過」→下界。前輪「現等級 2 建議降 3」撤回，改建議 1。</t>
         </is>
       </c>
       <c r="S29" s="2" t="inlineStr">
@@ -26193,7 +27137,7 @@
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
-          <t>只見搜尋摘錄 → 3 級</t>
+          <t>一手官方原文已讀（Andy 提供）→ 1 級；利害關係方須另有第二來源方可作基準（W1）</t>
         </is>
       </c>
     </row>
@@ -26630,31 +27574,31 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（artificialanalysis.ai 出口政策 CONNECT 403；非網站本身阻擋）；僅見搜尋摘要</t>
+          <t>R1 已讀原文（一手；1c 重讀：artificialanalysis.ai HTTP 200，網路已開放）</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>比較表列「Intelligence Index」：GPT-6 Sol (Max) 48｜GLM-5.3 (Max) 45；頁面註明 Index v4.3.2（10 項評測）</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>搜尋摘要：GPT-6 Sol（max）48、GLM-5.3（max）45</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>無需換算（頁面標示 Max 設定，與 SRC 一致）</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>一致（依搜尋摘要）</t>
+          <t>一致（值、版本 v4.3.2、設定 Max 皆相同）</t>
         </is>
       </c>
       <c r="N34" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -26673,7 +27617,7 @@
       </c>
       <c r="R34" s="2" t="inlineStr">
         <is>
-          <t>SRC 格敏感度 |ε|≈3.54（L1_Ans7，查核佇列第 1 名）：L1 前緣判定對 48／45 極敏感；第二批優先。摘要含 max 設定，SRC 對 GPT-6 Sol 未註明設定（需原文）</t>
+          <t>1c：由 R5→R1。S1 (a) 升級候選。頁面為即時快照，AA 可能修訂指數版本；日期以讀取日為準。敏感度最高（L1_Ans7，|ε|≈3.5），第二來源仍未查（單一評測機構；SemiAnalysis 規則不適用）。</t>
         </is>
       </c>
       <c r="S34" s="2" t="inlineStr">
@@ -26683,7 +27627,7 @@
       </c>
       <c r="T34" s="2" t="inlineStr">
         <is>
-          <t>只見搜尋摘錄 → 3 級</t>
+          <t>二手以外：一手網站原文已讀 → 1 級</t>
         </is>
       </c>
     </row>
@@ -26728,31 +27672,31 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（artificialanalysis.ai 出口政策 CONNECT 403；非網站本身阻擋）；僅見搜尋摘要</t>
+          <t>R1 已讀原文（一手；同頁）</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>同表同列：GLM-5.3 (Max) 45</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>搜尋摘要：GLM-5.3（max）45</t>
+          <t>45</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>無需換算</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>一致（依搜尋摘要）</t>
+          <t>一致</t>
         </is>
       </c>
       <c r="N35" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -26771,7 +27715,7 @@
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>SRC 格敏感度 |ε|≈3.54（L1_Ans7，查核佇列第 2 名）；第二批優先</t>
+          <t>1c：由 R5→R1。S1 (a) 升級候選。同 CAP_008。</t>
         </is>
       </c>
       <c r="S35" s="2" t="inlineStr">
@@ -26781,7 +27725,7 @@
       </c>
       <c r="T35" s="2" t="inlineStr">
         <is>
-          <t>只見搜尋摘錄 → 3 級</t>
+          <t>一手網站原文已讀 → 1 級</t>
         </is>
       </c>
     </row>
@@ -28078,7 +29022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -28457,6 +29401,91 @@
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>開放 artificialanalysis.ai 或由 Andy 另存比較頁</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>1c：SRC_HW_040 前輪「值不同」撤回</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>nvidia.com 規格表已讀：FP8 3,958 TFLOPS（含稀疏）；÷2＝1,979。</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>S1 (a) 升級候選（附換算式，標 Derived）；Spec_Rack C23／C40 說明文字可註明「含稀疏÷2」</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>1c：SRC_HW_014 出處更正與 F8／F10</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>227 kW 實為 NVIDIA 參考設計 MaxP（Schneider）；Supermicro 新聞稿無此數。F8 低 190 對 MaxQ 188、F10 高 230 對 MaxP 227。Spec_Rack F15 文字「Supermicro DLC-2 設計點 227 kW（S8）」不正確。</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>v5.18：SRC_HW_014 改引 Schneider（等級 1、Interested-party），F15 文字更正；F8／F10 是否改為 188／227 由 Project 決定</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>1c：SRC_DEM_011 升級</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Andy 讀官方原文（繁中頁）；值、「超過」、口徑、時點一致。</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>建議 1 級（立場 Interested-party）；是否需要英文原文由 Andy 決定</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>1c：SRC_CAP_008／011 升級</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>AA 頁面 R1，值 48／45 一致。</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>S1 (a) 升級候選；敏感度最高，建議另找第二指數（如 LMArena）作交叉</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>1c E2：Rubin Ultra 單架 72 GPU</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>詳見「1c E2 Rubin Ultra 單架72」。三項需判斷：(1)「GPU」＝封裝（推斷）或 die；(2) 單架功率區間 300–454 kW（無一手值）；(3) G28 取 72 或 576。價格無一手來源，只能維持 Assumed 推估 11.7／15.6／19.5 $M。</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Project 決定定義與各格；SRC_HW_054／013／045 改為 Kyber 備查或新增單架 SRC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stage 2-1d: W2 remaining re-verification, Supermicro/Schneider reads (read-only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017rvsjSzXV8yVCpbC82xsdQ
</commit_message>
<xml_diff>
--- a/docs/reports/20261005_stage2-1_查核.xlsx
+++ b/docs/reports/20261005_stage2-1_查核.xlsx
@@ -21,6 +21,7 @@
     <sheet name="1b 判讀與阻擋清單" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="1c 查核結果" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="1c E2 Rubin Ultra 單架72" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="1d 查核結果" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'查核紀錄'!$A$1:$T$30</definedName>
@@ -450,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -610,6 +611,18 @@
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>網路重測：artificialanalysis.ai HTTP 200、www.nvidia.com HTTP 307→200（非 403）。新增頁「1c 查核結果」「1c E2 Rubin Ultra 單架72」；更新「查核紀錄」（CAP_008／011、HW_040、HW_014、DEM_011）與「待 Project 判斷」。supermicro.com、flex.com、blog.se.com、prnewswire.com、storagereview.com、semianalysis.com 等仍為出口政策 CONNECT 403，未繞過。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1d（2026-10-05）</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>步驟 0：supermicro.com HTTP 302、blog.se.com HTTP 200（curl 通；supermicro 產品頁 curl 仍 Akamai 403，改以 WebFetch 讀成）。新增頁「1d 查核結果」；更新「查核紀錄」HW_003／004／005／006／010／014／015 與「待 Project 判斷」末 4 列。</t>
         </is>
       </c>
     </row>
@@ -22914,6 +22927,500 @@
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>依 Andy 決定不納入；Schneider 稱 Rubin Ultra＝Kyber 576 GPU／架、1–1.2 MW，與 NVIDIA 2026-09 衝突，列較舊路線圖，以 NVIDIA 為準</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>SRC_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>項目（值＋產品名）</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>讀取結果</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>原文摘錄（逐字，WebFetch／curl 取得）</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>實際所在頁面（網址）</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>前輪網址是否錯配</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>與現值</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>建議等級（G0-7）</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>立場與口徑（成本／售價）</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>備註</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_014 來源 2（Supermicro）</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Vera Rubin NVL72：DLC-2 “sized for 227 kW per rack”</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>R1（WebFetch 讀取頁面轉文字；curl 因 Akamai「Access Denied」403，同一網址須以 WebFetch 通道讀取）</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>“sized for 227 kW per rack”（WebFetch 回傳之逐字引文；搜尋結果摘要同句：“DLC-2 direct liquid cooling, from direct-to-chip cold plates through 1MW cooling towers, sized for 227 kW per rack”）</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.supermicro.com/en/accelerators/nvidia/vera-rubin</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>前輪：把摘要對應 ir.supermicro.com 新聞稿＝錯配（1c-3 已更正）。本輪網址＝摘要實際所在頁面</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>一致（227）</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>1（Interested-party，一手設備商）</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Supermicro（系統廠，賣方）。口徑＝DLC-2 液冷堆疊「sized for」每機架容量＝冷卻設計容量，非機架實測功率；WebFetch 的白話註解稱「power capacity」為其自行詮釋，原文只寫 sized for。</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>讀取通道限制：WebFetch 經小型模型轉文字，引文逐字但整頁上下文未逐行核對；與搜尋摘要兩條獨立通道句子相同。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_014 來源 1（Schneider）</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>VR NVL72：MaxP 227／MaxQ 188 kW/rack</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>R1（CC 環境自讀：curl HTTP 200；blog.se.com 已開放）</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>“Created for the NVIDIA Vera Rubin NVL72 racks, the validated reference design covers power and cooling and is integrated with Schneider Electric’s controls reference designs and supports operation at MaxQ 188 kw/rack and MaxP 227 kw/rack that delivers the most tokens.”</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://blog.se.com/datacenter/2026/05/08/nvidia-and-schneider-electric-get-in-sync-at-nvidia-gtc-2026-to-deliver-vera-rubin-ai-factories/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>不適用（本來源前輪即為正確頁面，且 chat 端已讀）；本輪取得 CC 自己的讀取紀錄</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>一致（F9＝227；F8 190 對 188；F10 230 對 227）</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>1（Interested-party）</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Schneider Electric（供電與冷卻設備商）。口徑＝NVIDIA VR NVL72 參考設計的機架 MaxP／MaxQ（IT 側）；日期取自網址路徑 2026-05-08，頁面本文未逐字列出日期。</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>兩來源（Supermicro 冷卻 sized-for、Schneider 參考設計 MaxP）數值同為 227，口徑不同，獨立性仍無法排除同源於 NVIDIA 參考設計。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_004（120–130）</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>GB200 NVL72 機架功率</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>120 端：R3（二手已讀，SemiAnalysis）；130 端：R5（未讀）</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>“This form factor requires approximately 120kW per rack”；“123.6kW per NVL72 is the total power draw including the inefficiencies from rectifying from AC power”（SemiAnalysis，WebFetch 回傳）</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://newsletter.semianalysis.com/p/gb200-hardware-architecture-and-component（120、123.6）；130：搜尋摘要稱 Gigabyte 頁 “up to 130 kW”，頁面 www.gigabyte.com/Enterprise/GIGAPOD-Pod-Scale/AI-DLC-POD_NVIDIA-GB200-NVL72 被出口政策擋（CONNECT 403），未讀；摘要稱 Supermicro 資料表 132 kW 電源架，PDF HTTP 503，未讀</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>錯配：前輪網址 moduledge.com／hashrateindex.com，兩者皆未讀到（moduledge 出口政策擋）；120 實際出現在 SemiAnalysis 頁</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>120：一致；130：未讀</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>120 端 2 級；整列仍 3（上緣 130 未讀原文）</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysis（付費研究機構，有訂閱誘因；G0-7 不得為唯一依據——本列僅此一個已讀來源，故不單獨升級）。口徑：120＝參考設計規格；123.6＝含 AC→DC 損耗的總用電；皆為 IT 側設計值，非 PUE 後設施電力。</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>模型 D9 基準 130、D8 低 120：已讀值 120／123.6 落在 120–130 內。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_005（132–142）</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>GB300 NVL72 機架功率</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>132–140：R3（二手已讀，wing.vc）；142：未讀</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>“It requires 132–140 kW of power”（wing.vc 摘要，WebFetch 回傳；原頁為 Data Gravity 文章轉載）</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wing.vc/content/how-much-does-an-nvidia-nvl72-cost</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>錯配：前輪網址 moduledge.com／hashrateindex.com 未讀（moduledge 出口政策擋）；132–140 實際出現在 wing.vc</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>132–140 一致；上緣 142 未見（頁面為 140）</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>整列 3；132–140 端 2 級</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>wing.vc（創投機構內容頁，非設備商；誘因＝內容行銷）。口徑未明（頁面未說 TDP 或最大）。搜尋摘要另稱 TDP 135、峰值 155（HPE 類），未讀。</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>現值上緣 142 高於已讀頁面 140：差 +1.4%，交 Project 判斷是否維持。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_003（220–320 千美元）</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>HGX H100 8-GPU 伺服器價格</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>R5／R6：無法把任何值對應到單一已讀頁面</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>（無；cyfuture.cloud 出口政策擋；其餘頁面未讀）</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>搜尋彙整摘要未標明逐項出處（出現的頁面：servermall.com、texas.gs.shi.com、vpsbenchmarks.com、cyfuture.cloud、electronics.alibaba.com），故不可為摘要指定網址；以「值＋產品名」反查（Arc Compute 6U HGX H100 起價 $210,000；ASUS ESC N8-E11/NV $249,200.05；7U 配置 $311,599.87）</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>錯配：前輪網址 clusterbid.com 未出現於任何反查結果，無法重現</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>摘要區間（21–32 萬）涵蓋現值；皆掛牌價，非成交價</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>經銷商掛牌價（銷售誘因）；口徑＝售價（掛牌），不含折讓</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>建議以「取得價區間」改記為「掛牌價」，由 Project 決定。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_006（2.8–3.4 百萬）</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>GB200 NVL72 機架價格</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>3.1：R3（二手已讀，wccftech）；2.8、3.4 端：未讀</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>“each such server rack currently costs around [$3.1 million]”（WebFetch 回傳，括號為其標示）；來源歸屬：文中引用 X 貼文 @firstadopter</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://wccftech.com/morgan-stanley-nvidia-gb200-nvl72-racks-deliver-a-profit-margin-of-77-6-vs-64-for-amd-mi355x-while-entailing-nearly-the-same-tco/amp/</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>錯配（歸屬）：前輪記「Morgan Stanley 3.1」；該頁的 3.1 並非 MS 估計，而是引用 X 貼文；前輪網址 Tom’s Hardware／Yahoo 未讀</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>3.1 一致（＝D12 基準）；2.8、3.4 端未讀</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>整列 3；3.1 端 2 級</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>wccftech（媒體）轉述個人貼文，方法未公開；口徑「currently costs」＝市價，成本或售價未明。</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>搜尋摘要另見：Wolfe Research（2026-01-30）約 3.0 M（GB200）與 4.3 M（GB300）；HSBC 報導約 3 M；「72 GPU 模組合計約 3.4 M」＝僅 GPU 模組，非整架，與 3.4 上緣口徑不同——皆為摘要，未讀。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_010（5.0 百萬）</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>GB300 NVL72 採購單價</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>R3（二手已讀，wing.vc）</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>“recent purchase orders reviewed in August 2026 show GB300 NVL72 racks priced at ‘just under $5.0M’ without cooling, or ‘~$32K more’ with an in-rack CDU”（wing.vc 摘要，WebFetch 回傳）；同頁：媒體估計 $6–6.5M</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.wing.vc/content/how-much-does-an-nvidia-nvl72-cost</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>否（前輪網址即此頁；本輪才讀到）</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>「略低於 5.0」對現值 5.0：值未逐字相同（差距未知，&lt;數%）；不含機架內 CDU</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2 級（二手已讀）；不構成 S1 (a) 升級（值非逐字相同）</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Data Gravity（經 wing.vc）；採購單成交價，口徑＝售價（買方付款），不含 CDU；原文 datagravity.dev 被出口政策擋，未讀</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>wing.vc 為轉載；同頁並列媒體 6–6.5 M，比現值高 20–30%。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SRC_HW_015（7.8 百萬）</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>VR200 NVL72 機架（Morgan Stanley）</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>R3（二手已讀，wccftech）</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>“a total estimated BOM of $7.8 million”（WebFetch 回傳）；頁面稱估計出自 Morgan Stanley Research；日期 2026-05-21；頁面無 Bernstein 數字</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://wccftech.com/nvidia-vera-rubin-rack-hit-with-memory-price-surge-pushing-hbm4-lpddr5x-bill-to-2m-of-7-8m-total/amp/（guru3d.com 同題報導 HTTP 403，未讀）</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>部分錯配：前輪列 Tom’s Hardware／PC Gamer／Guru3D／BigGo，已讀到者為 wccftech（前輪未列）；其餘頁面未讀</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>一致（7.8）</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2（二手已讀）</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Morgan Stanley Research（賣方研究，方法未公開）。**口徑＝BOM（物料成本），不是售價**；SRC 欄記「機架成本」一致，但 Spec_Rack 該列為「機架價格」。搜尋摘要另稱 “cost hyperscale cloud providers around $7.8 million per unit”（digitalcitizen.life，未讀）措辭近售價，與 BOM 衝突。</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Bernstein 9.1 M（HBM4 $53/GB）本輪未讀到原文，仍為摘要。</t>
         </is>
       </c>
     </row>
@@ -24766,7 +25273,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>moduledge.com；hashrateindex.com（SRC 登錄來源）</t>
+          <t>https://newsletter.semianalysis.com/p/gb200-hardware-architecture-and-component（120、123.6）；130：搜尋摘要稱 Gigabyte 頁 “up to 130 kW”，頁面 www.gigabyte.com/Enterprise/GIGAPOD-Pod-Scale/AI-DLC-POD_NVIDIA-GB200-NVL72 被出口政策擋（CONNECT 403），未讀；摘要稱 Supermicro 資料表 132 kW 電源架，PDF HTTP 503，未讀</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -24776,12 +25283,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（moduledge.com、hashrateindex.com、tomshardware.com 等 CONNECT 403）；僅見搜尋摘要</t>
+          <t>120 端：R3（二手已讀，SemiAnalysis）；130 端：R5（未讀）</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>“This form factor requires approximately 120kW per rack”；“123.6kW per NVL72 is the total power draw including the inefficiencies from rectifying from AC power”（SemiAnalysis，WebFetch 回傳）</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -24804,7 +25311,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>利害關係方：零組件／挖礦業者與系統廠，皆有銷售誘因</t>
+          <t>SemiAnalysis（付費研究機構，有訂閱誘因；G0-7 不得為唯一依據——本列僅此一個已讀來源，故不單獨升級）。口徑：120＝參考設計規格；123.6＝含 AC→DC 損耗的總用電；皆為 IT 側設計值，非 PUE 後設施電力。</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -24819,7 +25326,7 @@
       </c>
       <c r="R5" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取；四個值口徑不同的結論不變</t>
+          <t>重跑後無新增讀取；四個值口徑不同的結論不變 ｜1d：錯配：前輪網址 moduledge.com／hashrateindex.com，兩者皆未讀到（moduledge 出口政策擋）；120 實際出現在 SemiAnalysis 頁；模型 D9 基準 130、D8 低 120：已讀值 120／123.6 落在 120–130 內。</t>
         </is>
       </c>
       <c r="S5" s="2" t="inlineStr">
@@ -24864,7 +25371,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>moduledge.com；hashrateindex.com（SRC 登錄來源）</t>
+          <t>https://www.wing.vc/content/how-much-does-an-nvidia-nvl72-cost</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -24874,12 +25381,12 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（moduledge.com、hashrateindex.com、tomshardware.com 等 CONNECT 403）；僅見搜尋摘要</t>
+          <t>132–140：R3（二手已讀，wing.vc）；142：未讀</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>“It requires 132–140 kW of power”（wing.vc 摘要，WebFetch 回傳；原頁為 Data Gravity 文章轉載）</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -24902,7 +25409,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>利害關係方（零組件業者）；TrendForce 為研究機構（中立，估計值）</t>
+          <t>wing.vc（創投機構內容頁，非設備商；誘因＝內容行銷）。口徑未明（頁面未說 TDP 或最大）。搜尋摘要另稱 TDP 135、峰值 155（HPE 類），未讀。</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -24917,7 +25424,7 @@
       </c>
       <c r="R6" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取；四個值口徑不同的結論不變</t>
+          <t>重跑後無新增讀取；四個值口徑不同的結論不變 ｜1d：錯配：前輪網址 moduledge.com／hashrateindex.com 未讀（moduledge 出口政策擋）；132–140 實際出現在 wing.vc；現值上緣 142 高於已讀頁面 140：差 +1.4%，交 Project 判斷是否維持。</t>
         </is>
       </c>
       <c r="S6" s="2" t="inlineStr">
@@ -24962,7 +25469,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>https://blog.se.com/datacenter/2026/05/08/nvidia-and-schneider-electric-get-in-sync-at-nvidia-gtc-2026-to-deliver-vera-rubin-ai-factories/（Schneider Electric 部落格，2026-05-08；chat 端已讀原文）</t>
+          <t>https://blog.se.com/datacenter/2026/05/08/nvidia-and-schneider-electric-get-in-sync-at-nvidia-gtc-2026-to-deliver-vera-rubin-ai-factories/（Schneider Electric 部落格，2026-05-08；chat 端已讀原文）；Supermicro：https://www.supermicro.com/en/accelerators/nvidia/vera-rubin</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -24972,7 +25479,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R1 已讀原文（chat 端；CC 本環境 blog.se.com CONNECT 403，未獨立讀，依指令登錄；G2）</t>
+          <t>R1 已讀原文×2：Schneider（CC 本輪自讀，curl 200）；Supermicro 產品頁（WebFetch；curl 為 Akamai 403）</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -25015,7 +25522,7 @@
       </c>
       <c r="R7" s="2" t="inlineStr">
         <is>
-          <t>1c：原 SRC 記「Supermicro DLC-2 設計點」，經 Andy 讀新聞稿確認該稿無 227 kW；實際出處改為 Schneider 部落格（NVIDIA 參考設計 MaxP）。標籤文字（Spec_Rack F15「Supermicro DLC-2 設計點 227 kW（S8）」）需 v5.18 更正，屬判斷類，交 Project。CC 的搜尋摘要曾見 Supermicro 產品頁稱 “sized for 227 kW per rack”（supermicro.com 被擋，未讀原文，R5；僅旁證，不作依據）。查電源架備援配置之工作已取消。 更正（1c-3）：前輪把「sized for 227 kW per rack」摘要對應 ir.supermicro.com 新聞稿是錯配；新聞稿無此值（Andy 已讀），摘要所在頁面為 Supermicro 產品頁（上列網址）。</t>
+          <t>1c：原 SRC 記「Supermicro DLC-2 設計點」，經 Andy 讀新聞稿確認該稿無 227 kW；實際出處改為 Schneider 部落格（NVIDIA 參考設計 MaxP）。標籤文字（Spec_Rack F15「Supermicro DLC-2 設計點 227 kW（S8）」）需 v5.18 更正，屬判斷類，交 Project。CC 的搜尋摘要曾見 Supermicro 產品頁稱 “sized for 227 kW per rack”（supermicro.com 被擋，未讀原文，R5；僅旁證，不作依據）。查電源架備援配置之工作已取消。 更正（1c-3）：前輪把「sized for 227 kW per rack」摘要對應 ir.supermicro.com 新聞稿是錯配；新聞稿無此值（Andy 已讀），摘要所在頁面為 Supermicro 產品頁（上列網址）。 ｜1d：CC 環境已自行讀取兩頁，逐字引文見「1d 查核結果」；blog.se.com 與 supermicro.com 步驟 0 測得 HTTP 200／302。</t>
         </is>
       </c>
       <c r="S7" s="2" t="inlineStr">
@@ -25158,7 +25665,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>clusterbid.com（SRC 登錄；低品質來源）</t>
+          <t>搜尋彙整摘要未標明逐項出處（出現的頁面：servermall.com、texas.gs.shi.com、vpsbenchmarks.com、cyfuture.cloud、electronics.alibaba.com），故不可為摘要指定網址；以「值＋產品名」反查（Arc Compute 6U HGX H100 起價 $210,000；ASUS ESC N8-E11/NV $249,200.05；7U 配置 $311,599.87）</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -25168,12 +25675,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（clusterbid.com／tomshardware.com／wing.vc／pcgamer.com／guru3d.com CONNECT 403）；僅見搜尋摘要</t>
+          <t>R5／R6：無法把任何值對應到單一已讀頁面</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>（無；cyfuture.cloud 出口政策擋；其餘頁面未讀）</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -25196,7 +25703,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>利害關係方：經銷商掛牌價，有銷售誘因</t>
+          <t>經銷商掛牌價（銷售誘因）；口徑＝售價（掛牌），不含折讓</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -25211,7 +25718,7 @@
       </c>
       <c r="R9" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取</t>
+          <t>重跑後無新增讀取 ｜1d：錯配：前輪網址 clusterbid.com 未出現於任何反查結果，無法重現；建議以「取得價區間」改記為「掛牌價」，由 Project 決定。</t>
         </is>
       </c>
       <c r="S9" s="2" t="inlineStr">
@@ -25256,7 +25763,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Tom's Hardware（經 Yahoo Finance，SRC 登錄）</t>
+          <t>https://wccftech.com/morgan-stanley-nvidia-gb200-nvl72-racks-deliver-a-profit-margin-of-77-6-vs-64-for-amd-mi355x-while-entailing-nearly-the-same-tco/amp/</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -25266,12 +25773,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（clusterbid.com／tomshardware.com／wing.vc／pcgamer.com／guru3d.com CONNECT 403）；僅見搜尋摘要</t>
+          <t>3.1：R3（二手已讀，wccftech）；2.8、3.4 端：未讀</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>“each such server rack currently costs around [$3.1 million]”（WebFetch 回傳，括號為其標示）；來源歸屬：文中引用 X 貼文 @firstadopter</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -25294,7 +25801,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Wolfe、Morgan Stanley 為賣方研究（中立偏估計，方法未公開）；SemiAnalysis 另有付費訂閱誘因</t>
+          <t>wccftech（媒體）轉述個人貼文，方法未公開；口徑「currently costs」＝市價，成本或售價未明。</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -25309,7 +25816,7 @@
       </c>
       <c r="R10" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取</t>
+          <t>重跑後無新增讀取 ｜1d：錯配（歸屬）：前輪記「Morgan Stanley 3.1」；該頁的 3.1 並非 MS 估計，而是引用 X 貼文；前輪網址 Tom’s Hardware／Yahoo 未讀；搜尋摘要另見：Wolfe Research（2026-01-30）約 3.0 M（GB200）與 4.3 M（GB300）；HSBC 報導約 3 M；「72 GPU 模組合計約 3.4 M」＝僅 GPU 模組，非整架，與 3.4 上緣口徑不同——皆為摘要，未讀。</t>
         </is>
       </c>
       <c r="S10" s="2" t="inlineStr">
@@ -25354,7 +25861,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>https://www.wing.vc/content/how-much-does-an-nvidia-nvl72-cost（Data Gravity 經 wing.vc；SRC 登錄）</t>
+          <t>https://www.wing.vc/content/how-much-does-an-nvidia-nvl72-cost</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -25364,12 +25871,12 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（clusterbid.com／tomshardware.com／wing.vc／pcgamer.com／guru3d.com CONNECT 403）；僅見搜尋摘要</t>
+          <t>R3（二手已讀，wing.vc）</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>“recent purchase orders reviewed in August 2026 show GB300 NVL72 racks priced at ‘just under $5.0M’ without cooling, or ‘~$32K more’ with an in-rack CDU”（wing.vc 摘要，WebFetch 回傳）；同頁：媒體估計 $6–6.5M</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -25388,11 +25895,11 @@
         </is>
       </c>
       <c r="N11" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>利害關係方：未具名交易方，經 wing.vc／Data Gravity 轉述</t>
+          <t>Data Gravity（經 wing.vc）；採購單成交價，口徑＝售價（買方付款），不含 CDU；原文 datagravity.dev 被出口政策擋，未讀</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -25407,7 +25914,7 @@
       </c>
       <c r="R11" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取</t>
+          <t>重跑後無新增讀取 ｜1d：否（前輪網址即此頁；本輪才讀到）；wing.vc 為轉載；同頁並列媒體 6–6.5 M，比現值高 20–30%。</t>
         </is>
       </c>
       <c r="S11" s="2" t="inlineStr">
@@ -25452,7 +25959,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Tom's Hardware／PC Gamer／Guru3D 轉述 Morgan Stanley（SRC 登錄 PC Gamer、BigGo）</t>
+          <t>https://wccftech.com/nvidia-vera-rubin-rack-hit-with-memory-price-surge-pushing-hbm4-lpddr5x-bill-to-2m-of-7-8m-total/amp/（guru3d.com 同題報導 HTTP 403，未讀）</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -25462,12 +25969,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>R5 讀不到：被封鎖（clusterbid.com／tomshardware.com／wing.vc／pcgamer.com／guru3d.com CONNECT 403）；僅見搜尋摘要</t>
+          <t>R3（二手已讀，wccftech）</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>（未讀到原文，無可摘錄）</t>
+          <t>“a total estimated BOM of $7.8 million”（WebFetch 回傳）；頁面稱估計出自 Morgan Stanley Research；日期 2026-05-21；頁面無 Bernstein 數字</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -25486,11 +25993,11 @@
         </is>
       </c>
       <c r="N12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>中立（賣方研究，方法未公開）；SRC 現行標記為 IP（立場欄為中立）——兩者不一致，見待判斷</t>
+          <t>Morgan Stanley Research（賣方研究，方法未公開）。**口徑＝BOM（物料成本），不是售價**；SRC 欄記「機架成本」一致，但 Spec_Rack 該列為「機架價格」。搜尋摘要另稱 “cost hyperscale cloud providers around $7.8 million per unit”（digitalcitizen.life，未讀）措辭近售價，與 BOM 衝突。</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -25505,7 +26012,7 @@
       </c>
       <c r="R12" s="2" t="inlineStr">
         <is>
-          <t>重跑後無新增讀取</t>
+          <t>重跑後無新增讀取 ｜1d：部分錯配：前輪列 Tom’s Hardware／PC Gamer／Guru3D／BigGo，已讀到者為 wccftech（前輪未列）；其餘頁面未讀；Bernstein 9.1 M（HBM4 $53/GB）本輪未讀到原文，仍為摘要。</t>
         </is>
       </c>
       <c r="S12" s="2" t="inlineStr">
@@ -29066,7 +29573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -29547,6 +30054,74 @@
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>建議 v5.18 前由 CC 逐列複查 R5 網址與摘要對應（唯讀）；或指定先查哪幾列</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>1d：SRC_HW_015 口徑為成本（BOM）而非售價</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>已讀 wccftech：「total estimated BOM of $7.8 million」（Morgan Stanley Research）。Spec_Rack 為「機架價格」，若用於售價推導，成本與售價差（毛利）未計入</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>(a) 維持並於標籤註明「成本」；(b) 改查含毛利的售價來源（Bernstein 9.1 M 待讀）；(c) 以成本加毛利假設另立參數（判斷類）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>1d：SRC_HW_006 的 3.1 並非 Morgan Stanley 估計</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>已讀 wccftech：3.1 M 引自 X 貼文 @firstadopter；前輪記 Morgan Stanley 3.1 為錯配。3.4 上緣的搜尋摘要指「72 GPU 模組合計」，口徑不同</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>區間 2.8–3.4 的兩端皆無已讀原文；建議待讀 Tom’s Hardware 原文或改以 Wolfe 3.0／HSBC ≈3 等分析師值重定區間（判斷類）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>1d：SRC_HW_005 上緣 142 對已讀頁面 140；SRC_HW_004／005 的 130／142 端未讀</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>wing.vc 寫 132–140；SemiAnalysis 寫 120、123.6</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>維持現區間並註明已讀範圍；或上緣改 140（判斷類）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>1d：SRC_HW_014 兩來源口徑</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Supermicro＝DLC-2 冷卻 sized for 227；Schneider＝參考設計 MaxP 227，皆 CC 本環境已讀</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Spec_Rack F15 文字改記兩來源；獨立性仍無法排除同源 NVIDIA 參考設計</t>
         </is>
       </c>
     </row>

</xml_diff>